<commit_message>
chart folder repo update20260427
</commit_message>
<xml_diff>
--- a/MarketBullets_Master_Chart_Index.xlsx
+++ b/MarketBullets_Master_Chart_Index.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1efcf13b2cc8d9a/Documents/GitHub/WEBSITECHARTS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:9_{561CB34D-6201-43FF-BF1B-1FDB92941336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93C1E99C-D9FA-4DC3-9190-9FC24527930F}"/>
+  <xr:revisionPtr revIDLastSave="215" documentId="13_ncr:9_{561CB34D-6201-43FF-BF1B-1FDB92941336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A364967D-F527-4D51-A91B-CFDE64ABED06}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{0F0C2862-E87D-48A6-B1CD-4F9C66413518}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="368">
   <si>
     <t>Row #</t>
   </si>
@@ -61,9 +61,6 @@
     <t>Box-o-Rox Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_SRW_BOR_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Daily</t>
   </si>
   <si>
@@ -82,9 +79,6 @@
     <t>Chicago SRW 30-Minute</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_SRW_30M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>30-Min</t>
   </si>
   <si>
@@ -100,9 +94,6 @@
     <t>Chicago SRW Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_SRW_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Primary chart. Trend direction, moving averages, and daily close relative to BoR triggers.</t>
   </si>
   <si>
@@ -112,9 +103,6 @@
     <t>Chicago SRW Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_SRW_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Weekly</t>
   </si>
   <si>
@@ -127,9 +115,6 @@
     <t>Chicago SRW Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_SRW_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Monthly</t>
   </si>
   <si>
@@ -142,9 +127,6 @@
     <t>Chicago SRW Monthly (Annotated)</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_SRW_Special_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Longer-term pattern identification â€“ head-and-shoulders, channels, multi-year formations.</t>
   </si>
   <si>
@@ -154,9 +136,6 @@
     <t>Chicago SRW Annual</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_SRW_A.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Annual</t>
   </si>
   <si>
@@ -172,24 +151,15 @@
     <t>Kansas City HRW Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_HRW_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>In Development</t>
   </si>
   <si>
-    <t>HRW daily trend. Plains wheat quality premiums and basis implications for HRW producers.</t>
-  </si>
-  <si>
     <t>WHEAT_HRW_W.png</t>
   </si>
   <si>
     <t>Kansas City HRW Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_HRW_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Intermediate HRW trend. Relative strength vs SRW signals class rotation.</t>
   </si>
   <si>
@@ -199,33 +169,18 @@
     <t>Kansas City HRW Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_HRW_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
-    <t>HRW seasonal patterns. Winter wheat planting-to-harvest cycle visible here.</t>
-  </si>
-  <si>
     <t>WHEAT_HRS_D.png</t>
   </si>
   <si>
     <t>Minneapolis HRS Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_HRS_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
-    <t>Spring wheat daily. Protein premium dynamics and northern Plains weather sensitivity.</t>
-  </si>
-  <si>
     <t>WHEAT_HRS_W.png</t>
   </si>
   <si>
     <t>Minneapolis HRS Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_HRS_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>HRS intermediate trend. Spring planting window creates unique seasonal volatility.</t>
   </si>
   <si>
@@ -235,21 +190,12 @@
     <t>Minneapolis HRS Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_HRS_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
-    <t>HRS seasonal patterns. Protein premium cycles and milling demand trends.</t>
-  </si>
-  <si>
     <t>WHEAT_FWH_D.png</t>
   </si>
   <si>
     <t>Paris 11% Milling Wheat Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_FWH_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>European wheat benchmark. Black Sea export competition and EU crop conditions.</t>
   </si>
   <si>
@@ -259,9 +205,6 @@
     <t>Paris 11% Milling Wheat Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_FWH_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Global price discovery. Correlation to Chicago reveals export competitiveness shifts.</t>
   </si>
   <si>
@@ -271,12 +214,6 @@
     <t>Paris 11% Milling Wheat Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/WHEAT_FWH_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
-    <t>European wheat seasonal patterns. Northern hemisphere harvest overlap visible.</t>
-  </si>
-  <si>
     <t>GRAINS</t>
   </si>
   <si>
@@ -286,9 +223,6 @@
     <t>CBOT Corn Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/GRAIN_C_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Feed substitution and row crop bellwether.</t>
   </si>
   <si>
@@ -301,9 +235,6 @@
     <t>CBOT Corn Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/GRAIN_C_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Corn intermediate trend.</t>
   </si>
   <si>
@@ -313,9 +244,6 @@
     <t>CBOT Soybeans Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/GRAIN_S_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Row crop bellwether.</t>
   </si>
   <si>
@@ -325,9 +253,6 @@
     <t>CBOT Soybeans Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/GRAIN_S_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Soybean intermediate trend.</t>
   </si>
   <si>
@@ -340,9 +265,6 @@
     <t>Chicago SRW Spread: Mar/May</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_SRW_H_K.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Near-term carry.</t>
   </si>
   <si>
@@ -352,9 +274,6 @@
     <t>Chicago SRW Spread: May/Jul</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_SRW_K_N.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Pre-harvest carry signal.</t>
   </si>
   <si>
@@ -364,9 +283,6 @@
     <t>Chicago SRW Spread: Jul/Sep</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_SRW_N_U.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Harvest pressure spread.</t>
   </si>
   <si>
@@ -376,9 +292,6 @@
     <t>Chicago SRW Spread: Sep/Dec</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_SRW_U_Z.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Post-harvest carry.</t>
   </si>
   <si>
@@ -388,9 +301,6 @@
     <t>Chicago SRW Spread: Dec/Mar+1yr</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_SRW_Z_H2.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Winter carry.</t>
   </si>
   <si>
@@ -400,9 +310,6 @@
     <t>Kansas City HRW Spread: Mar/May</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_HRW_H_K.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>HRW near-term carry.</t>
   </si>
   <si>
@@ -412,9 +319,6 @@
     <t>Kansas City HRW Spread: May/Jul</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_HRW_K_N.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>HRW pre-harvest.</t>
   </si>
   <si>
@@ -424,9 +328,6 @@
     <t>Kansas City HRW Spread: Jul/Sep</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_HRW_N_U.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>HRW harvest-to-fall.</t>
   </si>
   <si>
@@ -436,9 +337,6 @@
     <t>Kansas City HRW Spread: Sep/Dec</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_HRW_U_Z.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>HRW fall carry.</t>
   </si>
   <si>
@@ -448,9 +346,6 @@
     <t>Kansas City HRW Spread: Dec/Mar+1yr</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_HRW_Z_H2.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>HRW winter carry.</t>
   </si>
   <si>
@@ -460,9 +355,6 @@
     <t>Minneapolis HRS Spread: Mar/May</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_HRS_H_K.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>HRS near-term carry.</t>
   </si>
   <si>
@@ -472,9 +364,6 @@
     <t>Minneapolis HRS Spread: May/Jul</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_HRS_K_N.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>HRS pre-harvest.</t>
   </si>
   <si>
@@ -484,9 +373,6 @@
     <t>Minneapolis HRS Spread: Jul/Sep</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_HRS_N_U.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>HRS harvest-to-fall.</t>
   </si>
   <si>
@@ -496,9 +382,6 @@
     <t>Minneapolis HRS Spread: Sep/Dec</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_HRS_U_Z.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>HRS fall carry.</t>
   </si>
   <si>
@@ -508,9 +391,6 @@
     <t>Minneapolis HRS Spread: Dec/Mar+1yr</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_HRS_Z_H2.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>HRS winter carry.</t>
   </si>
   <si>
@@ -520,9 +400,6 @@
     <t>Paris Milling Spread: Mar/May</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_FWH_H_K.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>European pre-harvest.</t>
   </si>
   <si>
@@ -532,9 +409,6 @@
     <t>Paris Milling Spread: May/Sep</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_FWH_K_U.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>European pre-harvest carry.</t>
   </si>
   <si>
@@ -544,9 +418,6 @@
     <t>Paris Milling Spread: May+1/Sep+1</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_FWH_K2_U2.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Unknown</t>
   </si>
   <si>
@@ -559,9 +430,6 @@
     <t>Paris Milling Spread: Sep/Dec</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_FWH_U_Z.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>European fall carry.</t>
   </si>
   <si>
@@ -571,9 +439,6 @@
     <t>Paris Milling Spread: Dec/Mar+1yr</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPD_FWH_Z_H2.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>European winter carry.</t>
   </si>
   <si>
@@ -586,9 +451,6 @@
     <t>Chicago SRW vs Kansas City HRW</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPDINTER_SRW_HRW_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Class premium/discount.</t>
   </si>
   <si>
@@ -601,9 +463,6 @@
     <t>Chicago SRW vs Minneapolis HRS</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPDINTER_SRW_HRS_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Protein premium.</t>
   </si>
   <si>
@@ -613,9 +472,6 @@
     <t>Chicago SRW vs Minneapolis HRS (Weekly)</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPDINTER_SRW_HRS_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Protein premium â€“ weekly.</t>
   </si>
   <si>
@@ -625,39 +481,15 @@
     <t>Minneapolis HRS vs Kansas City HRW</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPDINTER_HRS_HRW_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Quality differential.</t>
   </si>
   <si>
-    <t>SPDINTER_FWH_HRW_W.png</t>
-  </si>
-  <si>
     <t>Paris Milling vs Kansas City HRW (Weekly)</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPDINTER_FWH_HRW_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
-    <t>European vs US HRW â€“ weekly. ADDED: in repo but absent from prior indexes.</t>
-  </si>
-  <si>
-    <t>SPDINTER_FWH_HRW_M.png</t>
-  </si>
-  <si>
     <t>Paris Milling vs Kansas City HRW (Monthly)</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/SPDINTER_FWH_HRW_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
-    <t>Missing â€“ Not in Repo</t>
-  </si>
-  <si>
-    <t>File not yet exported/synced. Snippet ready for when file is added.</t>
-  </si>
-  <si>
     <t>RATIO</t>
   </si>
   <si>
@@ -667,9 +499,6 @@
     <t>Wheat/Corn Ratio: Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/RATIO_SRW_C_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Substitution economics.</t>
   </si>
   <si>
@@ -682,9 +511,6 @@
     <t>Soybeans/Corn Ratio: Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/RATIO_S_C_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Planting decision ratio.</t>
   </si>
   <si>
@@ -697,9 +523,6 @@
     <t>Commitment of Traders: Chicago SRW</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/COT_SRW_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Managed money positioning.</t>
   </si>
   <si>
@@ -709,9 +532,6 @@
     <t>Commitment of Traders: Kansas City HRW</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/COT_HRW_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>HRW positioning.</t>
   </si>
   <si>
@@ -724,9 +544,6 @@
     <t>2-Year T-Note Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/BNDS_2YR_TNOTE_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Near-term rate expectations.</t>
   </si>
   <si>
@@ -736,9 +553,6 @@
     <t>10-Year Treasury Bond Price: Quarterly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/BNDS_10YR_Price_Q.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Quarterly</t>
   </si>
   <si>
@@ -751,9 +565,6 @@
     <t>30-Year Treasury Bond Price: Quarterly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/BNDS_30YR_Price_Q.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Flight to quality signal.</t>
   </si>
   <si>
@@ -763,9 +574,6 @@
     <t>30-Year Treasury Bond Yield: Quarterly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/BNDS_30YR_Yield_Q.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Long-term borrowing cost.</t>
   </si>
   <si>
@@ -778,9 +586,6 @@
     <t>Australian Dollar Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/FX_WD_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Competitor currency (AUD). CORRECTED: prior index had FX_USD_WD_D.png â€“ repo filename is FX_WD_D.png.</t>
   </si>
   <si>
@@ -790,9 +595,6 @@
     <t>Australian Dollar Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/FX_WD_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Long-term AUD trend. CORRECTED: prior index had FX_USD_WD_M.png â€“ repo filename is FX_WD_M.png.</t>
   </si>
   <si>
@@ -802,9 +604,6 @@
     <t>Russian Rubles per US Dollar: Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/FX_RUB_USD_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Russian export competitiveness.</t>
   </si>
   <si>
@@ -814,9 +613,6 @@
     <t>Chinese Yuan per US Dollar: Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/FX_CNY_USD_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>China trade dynamics.</t>
   </si>
   <si>
@@ -826,9 +622,6 @@
     <t>Russian Rubles per Chinese Yuan: Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/FX_RUB_CNY_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Black Sea-China corridor.</t>
   </si>
   <si>
@@ -841,9 +634,6 @@
     <t>Crude Oil: Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/NRG_CL_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Energy trend.</t>
   </si>
   <si>
@@ -853,9 +643,6 @@
     <t>Crude Oil: Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/NRG_CL_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Energy trend â€“ weekly. ADDED: in repo but absent from prior indexes.</t>
   </si>
   <si>
@@ -865,9 +652,6 @@
     <t>Diesel/Heating Oil Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/NRG_HO_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Input cost â€“ immediate.</t>
   </si>
   <si>
@@ -877,9 +661,6 @@
     <t>Natural Gas: Henry Hub Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/NRG_NG_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Fertilizer feedstock.</t>
   </si>
   <si>
@@ -892,9 +673,6 @@
     <t>Gold (COMEX) Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/METL_GC_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Risk sentiment â€“ immediate.</t>
   </si>
   <si>
@@ -904,9 +682,6 @@
     <t>Gold (COMEX) Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/METL_GC_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Long-term risk gauge.</t>
   </si>
   <si>
@@ -916,9 +691,6 @@
     <t>Silver (COMEX) Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/METL_SI_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Industrial/monetary hybrid.</t>
   </si>
   <si>
@@ -928,9 +700,6 @@
     <t>Copper (COMEX) Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/METL_HG_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Dr. Copper â€“ economist's metal.</t>
   </si>
   <si>
@@ -943,9 +712,6 @@
     <t>US Dollar Index Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/IDX_DXY_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Currency impact.</t>
   </si>
   <si>
@@ -955,9 +721,6 @@
     <t>US Dollar Index Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/IDX_DXY_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Dollar long-term trend. STATUS UPDATED: file confirmed in repo â€“ was incorrectly marked In Development.</t>
   </si>
   <si>
@@ -967,9 +730,6 @@
     <t>Baltic Dry Index (Bulk Freight) Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/IDX_BDI_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Shipping costs.</t>
   </si>
   <si>
@@ -979,9 +739,6 @@
     <t>S&amp;P 500 Index Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/IDX_ES_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Risk appetite.</t>
   </si>
   <si>
@@ -991,9 +748,6 @@
     <t>S&amp;P 500 Index Monthly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/IDX_ES_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Equity trend.</t>
   </si>
   <si>
@@ -1003,9 +757,6 @@
     <t>Goldman Sachs Commodity Index Weekly</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/IDX_GSCI_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Commodity complex barometer.</t>
   </si>
   <si>
@@ -1018,9 +769,6 @@
     <t>John Deere &amp; Co. Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/FIN_DE_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Farm economy bellwether.</t>
   </si>
   <si>
@@ -1030,9 +778,6 @@
     <t>The Home Depot Daily</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/FIN_HD_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>Consumer strength proxy.</t>
   </si>
   <si>
@@ -1045,9 +790,6 @@
     <t>Unknown/Crypto</t>
   </si>
   <si>
-    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/MISC_CC_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
-  </si>
-  <si>
     <t>EXTRA â€“ needs documentation. Identify and assign category.</t>
   </si>
   <si>
@@ -1067,6 +809,321 @@
   </si>
   <si>
     <t>Needs Review:</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_SRW_BOR_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_SRW_30M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_SRW_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_SRW_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_SRW_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_SRW_Special_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_SRW_A.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_HRW_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_HRW_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_HRW_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_HRS_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_HRS_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_HRS_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_FWH_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_FWH_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/WHEAT_FWH_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/GRAIN_C_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/GRAIN_C_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/GRAIN_S_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/GRAIN_S_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_SRW_H_K.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_SRW_K_N.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_SRW_N_U.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_SRW_U_Z.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_SRW_Z_H2.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_HRW_H_K.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_HRW_K_N.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_HRW_N_U.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_HRW_U_Z.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_HRW_Z_H2.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_HRS_H_K.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_HRS_K_N.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_HRS_N_U.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_HRS_U_Z.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_HRS_Z_H2.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_FWH_H_K.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_FWH_K_U.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_FWH_K2_U2.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_FWH_U_Z.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPD_FWH_Z_H2.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPDINTER_SRW_HRW_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPDINTER_SRW_HRS_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPDINTER_SRW_HRS_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPDINTER_HRS_HRW_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPDINTER_HRW_FWH_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/SPDINTER_HRW_FWH_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/RATIO_SRW_C_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/RATIO_S_C_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/COT_SRW_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/COT_HRW_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/BNDS_2YR_TNOTE_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/BNDS_10YR_Price_Q.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/BNDS_30YR_Price_Q.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/BNDS_30YR_Yield_Q.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/FX_WD_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/FX_WD_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/FX_RUB_USD_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/FX_CNY_USD_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/FX_RUB_CNY_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/NRG_CL_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/NRG_CL_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/NRG_HO_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/NRG_NG_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/METL_GC_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/METL_GC_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/METL_SI_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/METL_HG_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/IDX_DXY_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/IDX_DXY_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/IDX_BDI_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/IDX_ES_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/IDX_ES_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/IDX_GSCI_W.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/FIN_DE_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/FIN_HD_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/MISC_CC_M.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>SPDINTER_HRW_FWH_W.png</t>
+  </si>
+  <si>
+    <t>RENAMED: was SPDINTER_FWH_HRW_W.png — corrected to match repo filename convention (HRW before FWH).</t>
+  </si>
+  <si>
+    <t>SPDINTER_HRW_FWH_M.png</t>
+  </si>
+  <si>
+    <t>RENAMED: was SPDINTER_FWH_HRW_M.png — corrected to match repo filename convention (HRW before FWH). File confirmed in repo.</t>
+  </si>
+  <si>
+    <t>FIN_ADM_D.png</t>
+  </si>
+  <si>
+    <t>Archer-Daniels-Midland Daily</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/FIN_ADM_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>ADDED: grain merchandising bellwether.</t>
+  </si>
+  <si>
+    <t>FIN_BG_D.png</t>
+  </si>
+  <si>
+    <t>Bunge Global Daily</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/FIN_BG_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>ADDED: global grain origination proxy.</t>
+  </si>
+  <si>
+    <t>FIN_CAT_D.png</t>
+  </si>
+  <si>
+    <t>Caterpillar Inc. Daily</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/FIN_CAT_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>ADDED: infrastructure / farm equipment demand proxy.</t>
+  </si>
+  <si>
+    <t>FIN_CHSCP_D.png</t>
+  </si>
+  <si>
+    <t>CHS Inc. Preferred Daily</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/FIN_CHSCP_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>ADDED: cooperative grain handler equity signal.</t>
+  </si>
+  <si>
+    <t>FIN_UNP_D.png</t>
+  </si>
+  <si>
+    <t>Union Pacific Railroad Daily</t>
+  </si>
+  <si>
+    <t>&lt;img src="https://raw.githubusercontent.com/MARKETBULLETSLLC/WEBSITECHARTS/main/charts/FIN_UNP_D.png" style="width:100%; display:block; margin:0; padding:0;" /&gt;</t>
+  </si>
+  <si>
+    <t>ADDED: grain rail transport bellwether.</t>
+  </si>
+  <si>
+    <t>HRW Daily — chart in development, not yet exported to repo.</t>
+  </si>
+  <si>
+    <t>HRW Monthly — chart in development, not yet exported to repo.</t>
+  </si>
+  <si>
+    <t>HRS Daily — chart in development, not yet exported to repo.</t>
+  </si>
+  <si>
+    <t>HRS Monthly — chart in development, not yet exported to repo.</t>
+  </si>
+  <si>
+    <t>FWH Monthly — chart in development, not yet exported to repo.</t>
   </si>
 </sst>
 </file>
@@ -1936,12 +1993,35 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="768" row="2">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{00427D8B-EFFB-4622-9B76-4838D824FA8D}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;8f793ef8-7004-451b-893d-aeaeda2bee1a&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D2140DC-1C2A-4E7F-919D-477AA469560B}">
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="46.85546875" customWidth="1"/>
+    <col min="5" max="5" width="175" customWidth="1"/>
     <col min="7" max="7" width="31" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1991,22 +2071,22 @@
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>263</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="I2" t="s">
-        <v>17</v>
-      </c>
       <c r="J2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -2017,28 +2097,28 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>264</v>
+      </c>
+      <c r="F3" t="s">
         <v>19</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" t="s">
         <v>20</v>
       </c>
-      <c r="F3" t="s">
+      <c r="I3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" t="s">
         <v>21</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -2049,28 +2129,28 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>265</v>
+      </c>
+      <c r="F4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="s">
         <v>24</v>
       </c>
-      <c r="D4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" t="s">
-        <v>27</v>
-      </c>
       <c r="I4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -2081,28 +2161,28 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" t="s">
         <v>28</v>
       </c>
-      <c r="D5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s">
-        <v>32</v>
-      </c>
       <c r="I5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J5" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -2113,28 +2193,28 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>267</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="I6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J6" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -2145,28 +2225,28 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>268</v>
       </c>
       <c r="F7" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="I7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J7" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -2177,28 +2257,28 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="E8" t="s">
-        <v>44</v>
+        <v>269</v>
       </c>
       <c r="F8" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H8" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="I8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J8" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -2209,28 +2289,28 @@
         <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="E9" t="s">
-        <v>50</v>
+        <v>270</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G9" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H9" t="s">
-        <v>52</v>
+        <v>363</v>
       </c>
       <c r="I9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -2241,28 +2321,28 @@
         <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="E10" t="s">
-        <v>55</v>
+        <v>271</v>
       </c>
       <c r="F10" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H10" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="I10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J10" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -2273,28 +2353,28 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>272</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G11" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H11" t="s">
-        <v>60</v>
+        <v>364</v>
       </c>
       <c r="I11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J11" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -2305,28 +2385,28 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="D12" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>273</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G12" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H12" t="s">
-        <v>64</v>
+        <v>365</v>
       </c>
       <c r="I12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -2337,28 +2417,28 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="D13" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="E13" t="s">
-        <v>67</v>
+        <v>274</v>
       </c>
       <c r="F13" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H13" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="I13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J13" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -2369,28 +2449,28 @@
         <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="E14" t="s">
-        <v>71</v>
+        <v>275</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G14" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H14" t="s">
-        <v>72</v>
+        <v>366</v>
       </c>
       <c r="I14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J14" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -2401,28 +2481,28 @@
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="D15" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="E15" t="s">
-        <v>75</v>
+        <v>276</v>
       </c>
       <c r="F15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H15" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="I15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -2433,28 +2513,28 @@
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="D16" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="E16" t="s">
-        <v>79</v>
+        <v>277</v>
       </c>
       <c r="F16" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H16" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="I16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J16" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -2465,28 +2545,28 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="E17" t="s">
-        <v>83</v>
+        <v>278</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G17" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H17" t="s">
-        <v>84</v>
+        <v>367</v>
       </c>
       <c r="I17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J17" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -2494,31 +2574,31 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="C18" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="D18" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="E18" t="s">
-        <v>88</v>
+        <v>279</v>
       </c>
       <c r="F18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H18" t="s">
-        <v>89</v>
+        <v>67</v>
       </c>
       <c r="I18" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -2526,31 +2606,31 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="C19" t="s">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="D19" t="s">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="E19" t="s">
-        <v>93</v>
+        <v>280</v>
       </c>
       <c r="F19" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H19" t="s">
-        <v>94</v>
+        <v>71</v>
       </c>
       <c r="I19" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J19" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -2558,31 +2638,31 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="C20" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="D20" t="s">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="E20" t="s">
-        <v>97</v>
+        <v>281</v>
       </c>
       <c r="F20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H20" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="I20" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -2590,31 +2670,31 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="C21" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="D21" t="s">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="E21" t="s">
-        <v>101</v>
+        <v>282</v>
       </c>
       <c r="F21" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H21" t="s">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="I21" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J21" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -2622,31 +2702,31 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C22" t="s">
-        <v>104</v>
+        <v>79</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="E22" t="s">
-        <v>106</v>
+        <v>283</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G22" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H22" t="s">
-        <v>107</v>
+        <v>81</v>
       </c>
       <c r="I22" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -2654,31 +2734,31 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C23" t="s">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="D23" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="E23" t="s">
-        <v>110</v>
+        <v>284</v>
       </c>
       <c r="F23" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H23" t="s">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="I23" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -2686,31 +2766,31 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C24" t="s">
-        <v>112</v>
+        <v>85</v>
       </c>
       <c r="D24" t="s">
-        <v>113</v>
+        <v>86</v>
       </c>
       <c r="E24" t="s">
-        <v>114</v>
+        <v>285</v>
       </c>
       <c r="F24" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H24" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="I24" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -2718,31 +2798,31 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C25" t="s">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="D25" t="s">
-        <v>117</v>
+        <v>89</v>
       </c>
       <c r="E25" t="s">
-        <v>118</v>
+        <v>286</v>
       </c>
       <c r="F25" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G25" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H25" t="s">
-        <v>119</v>
+        <v>90</v>
       </c>
       <c r="I25" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -2750,31 +2830,31 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C26" t="s">
-        <v>120</v>
+        <v>91</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>121</v>
+        <v>92</v>
       </c>
       <c r="E26" t="s">
-        <v>122</v>
+        <v>287</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G26" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H26" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="I26" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -2782,31 +2862,31 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C27" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
       <c r="E27" t="s">
-        <v>126</v>
+        <v>288</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G27" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H27" t="s">
-        <v>127</v>
+        <v>96</v>
       </c>
       <c r="I27" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -2814,31 +2894,31 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C28" t="s">
-        <v>128</v>
+        <v>97</v>
       </c>
       <c r="D28" t="s">
-        <v>129</v>
+        <v>98</v>
       </c>
       <c r="E28" t="s">
-        <v>130</v>
+        <v>289</v>
       </c>
       <c r="F28" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G28" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H28" t="s">
-        <v>131</v>
+        <v>99</v>
       </c>
       <c r="I28" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
@@ -2846,31 +2926,31 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C29" t="s">
-        <v>132</v>
+        <v>100</v>
       </c>
       <c r="D29" t="s">
-        <v>133</v>
+        <v>101</v>
       </c>
       <c r="E29" t="s">
-        <v>134</v>
+        <v>290</v>
       </c>
       <c r="F29" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H29" t="s">
-        <v>135</v>
+        <v>102</v>
       </c>
       <c r="I29" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
@@ -2878,31 +2958,31 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" t="s">
         <v>103</v>
       </c>
-      <c r="C30" t="s">
-        <v>136</v>
-      </c>
       <c r="D30" t="s">
-        <v>137</v>
+        <v>104</v>
       </c>
       <c r="E30" t="s">
-        <v>138</v>
+        <v>291</v>
       </c>
       <c r="F30" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G30" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H30" t="s">
-        <v>139</v>
+        <v>105</v>
       </c>
       <c r="I30" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
@@ -2910,31 +2990,31 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C31" t="s">
-        <v>140</v>
+        <v>106</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>141</v>
+        <v>107</v>
       </c>
       <c r="E31" t="s">
-        <v>142</v>
+        <v>292</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G31" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H31" t="s">
-        <v>143</v>
+        <v>108</v>
       </c>
       <c r="I31" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -2942,31 +3022,31 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C32" t="s">
-        <v>144</v>
+        <v>109</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>145</v>
+        <v>110</v>
       </c>
       <c r="E32" t="s">
-        <v>146</v>
+        <v>293</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G32" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H32" t="s">
-        <v>147</v>
+        <v>111</v>
       </c>
       <c r="I32" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
@@ -2974,31 +3054,31 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C33" t="s">
-        <v>148</v>
+        <v>112</v>
       </c>
       <c r="D33" t="s">
-        <v>149</v>
+        <v>113</v>
       </c>
       <c r="E33" t="s">
-        <v>150</v>
+        <v>294</v>
       </c>
       <c r="F33" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G33" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H33" t="s">
-        <v>151</v>
+        <v>114</v>
       </c>
       <c r="I33" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
@@ -3006,31 +3086,31 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C34" t="s">
-        <v>152</v>
+        <v>115</v>
       </c>
       <c r="D34" t="s">
-        <v>153</v>
+        <v>116</v>
       </c>
       <c r="E34" t="s">
-        <v>154</v>
+        <v>295</v>
       </c>
       <c r="F34" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G34" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H34" t="s">
-        <v>155</v>
+        <v>117</v>
       </c>
       <c r="I34" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J34" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
@@ -3038,31 +3118,31 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C35" t="s">
-        <v>156</v>
+        <v>118</v>
       </c>
       <c r="D35" t="s">
-        <v>157</v>
+        <v>119</v>
       </c>
       <c r="E35" t="s">
-        <v>158</v>
+        <v>296</v>
       </c>
       <c r="F35" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G35" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H35" t="s">
-        <v>159</v>
+        <v>120</v>
       </c>
       <c r="I35" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J35" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
@@ -3070,31 +3150,31 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C36" t="s">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>161</v>
+        <v>122</v>
       </c>
       <c r="E36" t="s">
-        <v>162</v>
+        <v>297</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G36" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H36" t="s">
-        <v>163</v>
+        <v>123</v>
       </c>
       <c r="I36" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J36" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -3102,31 +3182,31 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C37" t="s">
-        <v>164</v>
+        <v>124</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>165</v>
+        <v>125</v>
       </c>
       <c r="E37" t="s">
-        <v>166</v>
+        <v>298</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G37" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H37" t="s">
-        <v>167</v>
+        <v>126</v>
       </c>
       <c r="I37" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J37" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
@@ -3134,31 +3214,31 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C38" t="s">
-        <v>168</v>
+        <v>127</v>
       </c>
       <c r="D38" t="s">
-        <v>169</v>
+        <v>128</v>
       </c>
       <c r="E38" t="s">
-        <v>170</v>
+        <v>299</v>
       </c>
       <c r="F38" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G38" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H38" t="s">
-        <v>171</v>
+        <v>129</v>
       </c>
       <c r="I38" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J38" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
@@ -3166,31 +3246,31 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C39" t="s">
-        <v>172</v>
+        <v>130</v>
       </c>
       <c r="D39" t="s">
-        <v>173</v>
+        <v>131</v>
       </c>
       <c r="E39" t="s">
-        <v>174</v>
+        <v>300</v>
       </c>
       <c r="F39" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G39" t="s">
-        <v>175</v>
+        <v>132</v>
       </c>
       <c r="H39" t="s">
-        <v>176</v>
+        <v>133</v>
       </c>
       <c r="I39" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J39" t="s">
-        <v>175</v>
+        <v>132</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
@@ -3198,31 +3278,31 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C40" t="s">
-        <v>177</v>
+        <v>134</v>
       </c>
       <c r="D40" t="s">
-        <v>178</v>
+        <v>135</v>
       </c>
       <c r="E40" t="s">
-        <v>179</v>
+        <v>301</v>
       </c>
       <c r="F40" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G40" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H40" t="s">
-        <v>180</v>
+        <v>136</v>
       </c>
       <c r="I40" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J40" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
@@ -3230,31 +3310,31 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="C41" t="s">
-        <v>181</v>
+        <v>137</v>
       </c>
       <c r="D41" t="s">
-        <v>182</v>
+        <v>138</v>
       </c>
       <c r="E41" t="s">
-        <v>183</v>
+        <v>302</v>
       </c>
       <c r="F41" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G41" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H41" t="s">
-        <v>184</v>
+        <v>139</v>
       </c>
       <c r="I41" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J41" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
@@ -3262,31 +3342,31 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>185</v>
+        <v>140</v>
       </c>
       <c r="C42" t="s">
-        <v>186</v>
+        <v>141</v>
       </c>
       <c r="D42" t="s">
-        <v>187</v>
+        <v>142</v>
       </c>
       <c r="E42" t="s">
-        <v>188</v>
+        <v>303</v>
       </c>
       <c r="F42" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G42" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H42" t="s">
-        <v>189</v>
+        <v>143</v>
       </c>
       <c r="I42" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J42" t="s">
-        <v>190</v>
+        <v>144</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
@@ -3294,31 +3374,31 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>185</v>
+        <v>140</v>
       </c>
       <c r="C43" t="s">
-        <v>191</v>
+        <v>145</v>
       </c>
       <c r="D43" t="s">
-        <v>192</v>
+        <v>146</v>
       </c>
       <c r="E43" t="s">
-        <v>193</v>
+        <v>304</v>
       </c>
       <c r="F43" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H43" t="s">
-        <v>194</v>
+        <v>147</v>
       </c>
       <c r="I43" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J43" t="s">
-        <v>190</v>
+        <v>144</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -3326,31 +3406,31 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>185</v>
+        <v>140</v>
       </c>
       <c r="C44" t="s">
-        <v>195</v>
+        <v>148</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>196</v>
+        <v>149</v>
       </c>
       <c r="E44" t="s">
-        <v>197</v>
+        <v>305</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G44" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H44" t="s">
-        <v>198</v>
+        <v>150</v>
       </c>
       <c r="I44" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J44" t="s">
-        <v>190</v>
+        <v>144</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -3358,31 +3438,31 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>185</v>
+        <v>140</v>
       </c>
       <c r="C45" t="s">
-        <v>199</v>
+        <v>151</v>
       </c>
       <c r="D45" t="s">
-        <v>200</v>
+        <v>152</v>
       </c>
       <c r="E45" t="s">
-        <v>201</v>
+        <v>306</v>
       </c>
       <c r="F45" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G45" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H45" t="s">
-        <v>202</v>
+        <v>153</v>
       </c>
       <c r="I45" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J45" t="s">
-        <v>190</v>
+        <v>144</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
@@ -3390,31 +3470,31 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>185</v>
+        <v>140</v>
       </c>
       <c r="C46" t="s">
-        <v>203</v>
+        <v>339</v>
       </c>
       <c r="D46" t="s">
-        <v>204</v>
+        <v>154</v>
       </c>
       <c r="E46" t="s">
-        <v>205</v>
+        <v>307</v>
       </c>
       <c r="F46" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G46" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H46" t="s">
-        <v>206</v>
+        <v>340</v>
       </c>
       <c r="I46" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J46" t="s">
-        <v>190</v>
+        <v>144</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
@@ -3422,31 +3502,31 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>185</v>
+        <v>140</v>
       </c>
       <c r="C47" t="s">
-        <v>207</v>
+        <v>341</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>208</v>
+        <v>155</v>
       </c>
       <c r="E47" t="s">
-        <v>209</v>
+        <v>308</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G47" t="s">
-        <v>210</v>
+        <v>14</v>
       </c>
       <c r="H47" t="s">
-        <v>211</v>
+        <v>342</v>
       </c>
       <c r="I47" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J47" t="s">
-        <v>190</v>
+        <v>144</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
@@ -3454,31 +3534,31 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>212</v>
+        <v>156</v>
       </c>
       <c r="C48" t="s">
-        <v>213</v>
+        <v>157</v>
       </c>
       <c r="D48" t="s">
-        <v>214</v>
+        <v>158</v>
       </c>
       <c r="E48" t="s">
-        <v>215</v>
+        <v>309</v>
       </c>
       <c r="F48" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G48" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H48" t="s">
-        <v>216</v>
+        <v>159</v>
       </c>
       <c r="I48" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J48" t="s">
-        <v>190</v>
+        <v>144</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
@@ -3486,31 +3566,31 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>212</v>
+        <v>156</v>
       </c>
       <c r="C49" t="s">
-        <v>218</v>
+        <v>161</v>
       </c>
       <c r="D49" t="s">
-        <v>219</v>
+        <v>162</v>
       </c>
       <c r="E49" t="s">
-        <v>220</v>
+        <v>310</v>
       </c>
       <c r="F49" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H49" t="s">
-        <v>221</v>
+        <v>163</v>
       </c>
       <c r="I49" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J49" t="s">
-        <v>190</v>
+        <v>144</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
@@ -3518,31 +3598,31 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>222</v>
+        <v>164</v>
       </c>
       <c r="C50" t="s">
-        <v>223</v>
+        <v>165</v>
       </c>
       <c r="D50" t="s">
-        <v>224</v>
+        <v>166</v>
       </c>
       <c r="E50" t="s">
-        <v>225</v>
+        <v>311</v>
       </c>
       <c r="F50" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G50" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H50" t="s">
-        <v>226</v>
+        <v>167</v>
       </c>
       <c r="I50" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J50" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
@@ -3550,31 +3630,31 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>222</v>
+        <v>164</v>
       </c>
       <c r="C51" t="s">
-        <v>227</v>
+        <v>168</v>
       </c>
       <c r="D51" t="s">
-        <v>228</v>
+        <v>169</v>
       </c>
       <c r="E51" t="s">
-        <v>229</v>
+        <v>312</v>
       </c>
       <c r="F51" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G51" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H51" t="s">
-        <v>230</v>
+        <v>170</v>
       </c>
       <c r="I51" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="J51" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
@@ -3582,31 +3662,31 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>231</v>
+        <v>171</v>
       </c>
       <c r="C52" t="s">
-        <v>232</v>
+        <v>172</v>
       </c>
       <c r="D52" t="s">
-        <v>233</v>
+        <v>173</v>
       </c>
       <c r="E52" t="s">
-        <v>234</v>
+        <v>313</v>
       </c>
       <c r="F52" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G52" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H52" t="s">
-        <v>235</v>
+        <v>174</v>
       </c>
       <c r="I52" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J52" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
@@ -3614,31 +3694,31 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>231</v>
+        <v>171</v>
       </c>
       <c r="C53" t="s">
-        <v>236</v>
+        <v>175</v>
       </c>
       <c r="D53" t="s">
-        <v>237</v>
+        <v>176</v>
       </c>
       <c r="E53" t="s">
-        <v>238</v>
+        <v>314</v>
       </c>
       <c r="F53" t="s">
-        <v>239</v>
+        <v>177</v>
       </c>
       <c r="G53" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H53" t="s">
-        <v>240</v>
+        <v>178</v>
       </c>
       <c r="I53" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J53" t="s">
-        <v>239</v>
+        <v>177</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
@@ -3646,31 +3726,31 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>231</v>
+        <v>171</v>
       </c>
       <c r="C54" t="s">
-        <v>241</v>
+        <v>179</v>
       </c>
       <c r="D54" t="s">
-        <v>242</v>
+        <v>180</v>
       </c>
       <c r="E54" t="s">
-        <v>243</v>
+        <v>315</v>
       </c>
       <c r="F54" t="s">
-        <v>239</v>
+        <v>177</v>
       </c>
       <c r="G54" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H54" t="s">
-        <v>244</v>
+        <v>181</v>
       </c>
       <c r="I54" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J54" t="s">
-        <v>239</v>
+        <v>177</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
@@ -3678,31 +3758,31 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>231</v>
+        <v>171</v>
       </c>
       <c r="C55" t="s">
-        <v>245</v>
+        <v>182</v>
       </c>
       <c r="D55" t="s">
-        <v>246</v>
+        <v>183</v>
       </c>
       <c r="E55" t="s">
-        <v>247</v>
+        <v>316</v>
       </c>
       <c r="F55" t="s">
-        <v>239</v>
+        <v>177</v>
       </c>
       <c r="G55" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H55" t="s">
-        <v>248</v>
+        <v>184</v>
       </c>
       <c r="I55" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J55" t="s">
-        <v>239</v>
+        <v>177</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
@@ -3710,31 +3790,31 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>249</v>
+        <v>185</v>
       </c>
       <c r="C56" t="s">
-        <v>250</v>
+        <v>186</v>
       </c>
       <c r="D56" t="s">
-        <v>251</v>
+        <v>187</v>
       </c>
       <c r="E56" t="s">
-        <v>252</v>
+        <v>317</v>
       </c>
       <c r="F56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G56" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H56" t="s">
-        <v>253</v>
+        <v>188</v>
       </c>
       <c r="I56" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
@@ -3742,31 +3822,31 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>249</v>
+        <v>185</v>
       </c>
       <c r="C57" t="s">
-        <v>254</v>
+        <v>189</v>
       </c>
       <c r="D57" t="s">
-        <v>255</v>
+        <v>190</v>
       </c>
       <c r="E57" t="s">
-        <v>256</v>
+        <v>318</v>
       </c>
       <c r="F57" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G57" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H57" t="s">
-        <v>257</v>
+        <v>191</v>
       </c>
       <c r="I57" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J57" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
@@ -3774,31 +3854,31 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>249</v>
+        <v>185</v>
       </c>
       <c r="C58" t="s">
-        <v>258</v>
+        <v>192</v>
       </c>
       <c r="D58" t="s">
-        <v>259</v>
+        <v>193</v>
       </c>
       <c r="E58" t="s">
-        <v>260</v>
+        <v>319</v>
       </c>
       <c r="F58" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G58" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H58" t="s">
-        <v>261</v>
+        <v>194</v>
       </c>
       <c r="I58" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J58" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
@@ -3806,31 +3886,31 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>249</v>
+        <v>185</v>
       </c>
       <c r="C59" t="s">
-        <v>262</v>
+        <v>195</v>
       </c>
       <c r="D59" t="s">
-        <v>263</v>
+        <v>196</v>
       </c>
       <c r="E59" t="s">
-        <v>264</v>
+        <v>320</v>
       </c>
       <c r="F59" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G59" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H59" t="s">
-        <v>265</v>
+        <v>197</v>
       </c>
       <c r="I59" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J59" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
@@ -3838,31 +3918,31 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>249</v>
+        <v>185</v>
       </c>
       <c r="C60" t="s">
-        <v>266</v>
+        <v>198</v>
       </c>
       <c r="D60" t="s">
-        <v>267</v>
+        <v>199</v>
       </c>
       <c r="E60" t="s">
-        <v>268</v>
+        <v>321</v>
       </c>
       <c r="F60" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G60" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H60" t="s">
-        <v>269</v>
+        <v>200</v>
       </c>
       <c r="I60" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J60" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
@@ -3870,31 +3950,31 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>270</v>
+        <v>201</v>
       </c>
       <c r="C61" t="s">
-        <v>271</v>
+        <v>202</v>
       </c>
       <c r="D61" t="s">
-        <v>272</v>
+        <v>203</v>
       </c>
       <c r="E61" t="s">
-        <v>273</v>
+        <v>322</v>
       </c>
       <c r="F61" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G61" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H61" t="s">
-        <v>274</v>
+        <v>204</v>
       </c>
       <c r="I61" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J61" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
@@ -3902,31 +3982,31 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>270</v>
+        <v>201</v>
       </c>
       <c r="C62" t="s">
-        <v>275</v>
+        <v>205</v>
       </c>
       <c r="D62" t="s">
-        <v>276</v>
+        <v>206</v>
       </c>
       <c r="E62" t="s">
-        <v>277</v>
+        <v>323</v>
       </c>
       <c r="F62" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G62" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H62" t="s">
-        <v>278</v>
+        <v>207</v>
       </c>
       <c r="I62" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J62" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
@@ -3934,31 +4014,31 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>270</v>
+        <v>201</v>
       </c>
       <c r="C63" t="s">
-        <v>279</v>
+        <v>208</v>
       </c>
       <c r="D63" t="s">
-        <v>280</v>
+        <v>209</v>
       </c>
       <c r="E63" t="s">
-        <v>281</v>
+        <v>324</v>
       </c>
       <c r="F63" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G63" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H63" t="s">
-        <v>282</v>
+        <v>210</v>
       </c>
       <c r="I63" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J63" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
@@ -3966,31 +4046,31 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>270</v>
+        <v>201</v>
       </c>
       <c r="C64" t="s">
-        <v>283</v>
+        <v>211</v>
       </c>
       <c r="D64" t="s">
-        <v>284</v>
+        <v>212</v>
       </c>
       <c r="E64" t="s">
-        <v>285</v>
+        <v>325</v>
       </c>
       <c r="F64" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G64" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H64" t="s">
-        <v>286</v>
+        <v>213</v>
       </c>
       <c r="I64" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J64" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
@@ -3998,31 +4078,31 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>287</v>
+        <v>214</v>
       </c>
       <c r="C65" t="s">
-        <v>288</v>
+        <v>215</v>
       </c>
       <c r="D65" t="s">
-        <v>289</v>
+        <v>216</v>
       </c>
       <c r="E65" t="s">
-        <v>290</v>
+        <v>326</v>
       </c>
       <c r="F65" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G65" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H65" t="s">
-        <v>291</v>
+        <v>217</v>
       </c>
       <c r="I65" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J65" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
@@ -4030,31 +4110,31 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>287</v>
+        <v>214</v>
       </c>
       <c r="C66" t="s">
-        <v>292</v>
+        <v>218</v>
       </c>
       <c r="D66" t="s">
-        <v>293</v>
+        <v>219</v>
       </c>
       <c r="E66" t="s">
-        <v>294</v>
+        <v>327</v>
       </c>
       <c r="F66" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G66" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H66" t="s">
-        <v>295</v>
+        <v>220</v>
       </c>
       <c r="I66" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J66" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
@@ -4062,31 +4142,31 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>287</v>
+        <v>214</v>
       </c>
       <c r="C67" t="s">
-        <v>296</v>
+        <v>221</v>
       </c>
       <c r="D67" t="s">
-        <v>297</v>
+        <v>222</v>
       </c>
       <c r="E67" t="s">
-        <v>298</v>
+        <v>328</v>
       </c>
       <c r="F67" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G67" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H67" t="s">
-        <v>299</v>
+        <v>223</v>
       </c>
       <c r="I67" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J67" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
@@ -4094,31 +4174,31 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>287</v>
+        <v>214</v>
       </c>
       <c r="C68" t="s">
-        <v>300</v>
+        <v>224</v>
       </c>
       <c r="D68" t="s">
-        <v>301</v>
+        <v>225</v>
       </c>
       <c r="E68" t="s">
-        <v>302</v>
+        <v>329</v>
       </c>
       <c r="F68" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G68" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H68" t="s">
-        <v>303</v>
+        <v>226</v>
       </c>
       <c r="I68" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J68" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
@@ -4126,31 +4206,31 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>304</v>
+        <v>227</v>
       </c>
       <c r="C69" t="s">
-        <v>305</v>
+        <v>228</v>
       </c>
       <c r="D69" t="s">
-        <v>306</v>
+        <v>229</v>
       </c>
       <c r="E69" t="s">
-        <v>307</v>
+        <v>330</v>
       </c>
       <c r="F69" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G69" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H69" t="s">
-        <v>308</v>
+        <v>230</v>
       </c>
       <c r="I69" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J69" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
@@ -4158,31 +4238,31 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>304</v>
+        <v>227</v>
       </c>
       <c r="C70" t="s">
-        <v>309</v>
+        <v>231</v>
       </c>
       <c r="D70" t="s">
-        <v>310</v>
+        <v>232</v>
       </c>
       <c r="E70" t="s">
-        <v>311</v>
+        <v>331</v>
       </c>
       <c r="F70" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G70" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H70" t="s">
-        <v>312</v>
+        <v>233</v>
       </c>
       <c r="I70" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J70" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
@@ -4190,31 +4270,31 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>304</v>
+        <v>227</v>
       </c>
       <c r="C71" t="s">
-        <v>313</v>
+        <v>234</v>
       </c>
       <c r="D71" t="s">
-        <v>314</v>
+        <v>235</v>
       </c>
       <c r="E71" t="s">
-        <v>315</v>
+        <v>332</v>
       </c>
       <c r="F71" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G71" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H71" t="s">
-        <v>316</v>
+        <v>236</v>
       </c>
       <c r="I71" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J71" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
@@ -4222,31 +4302,31 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>304</v>
+        <v>227</v>
       </c>
       <c r="C72" t="s">
-        <v>317</v>
+        <v>237</v>
       </c>
       <c r="D72" t="s">
-        <v>318</v>
+        <v>238</v>
       </c>
       <c r="E72" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
       <c r="F72" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G72" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H72" t="s">
-        <v>320</v>
+        <v>239</v>
       </c>
       <c r="I72" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J72" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
@@ -4254,31 +4334,31 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>304</v>
+        <v>227</v>
       </c>
       <c r="C73" t="s">
-        <v>321</v>
+        <v>240</v>
       </c>
       <c r="D73" t="s">
-        <v>322</v>
+        <v>241</v>
       </c>
       <c r="E73" t="s">
-        <v>323</v>
+        <v>334</v>
       </c>
       <c r="F73" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G73" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H73" t="s">
-        <v>324</v>
+        <v>242</v>
       </c>
       <c r="I73" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J73" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
@@ -4286,31 +4366,31 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>304</v>
+        <v>227</v>
       </c>
       <c r="C74" t="s">
-        <v>325</v>
+        <v>243</v>
       </c>
       <c r="D74" t="s">
-        <v>326</v>
+        <v>244</v>
       </c>
       <c r="E74" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="F74" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G74" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H74" t="s">
-        <v>328</v>
+        <v>245</v>
       </c>
       <c r="I74" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J74" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
@@ -4318,31 +4398,31 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>329</v>
+        <v>246</v>
       </c>
       <c r="C75" t="s">
-        <v>330</v>
+        <v>247</v>
       </c>
       <c r="D75" t="s">
-        <v>331</v>
+        <v>248</v>
       </c>
       <c r="E75" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="F75" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G75" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H75" t="s">
-        <v>333</v>
+        <v>249</v>
       </c>
       <c r="I75" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J75" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
@@ -4350,31 +4430,31 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>329</v>
+        <v>246</v>
       </c>
       <c r="C76" t="s">
-        <v>334</v>
+        <v>250</v>
       </c>
       <c r="D76" t="s">
-        <v>335</v>
+        <v>251</v>
       </c>
       <c r="E76" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F76" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G76" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H76" t="s">
-        <v>337</v>
+        <v>252</v>
       </c>
       <c r="I76" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="J76" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
@@ -4382,79 +4462,239 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
+        <v>246</v>
+      </c>
+      <c r="C77" t="s">
+        <v>343</v>
+      </c>
+      <c r="D77" t="s">
+        <v>344</v>
+      </c>
+      <c r="E77" t="s">
+        <v>345</v>
+      </c>
+      <c r="F77" t="s">
+        <v>13</v>
+      </c>
+      <c r="G77" t="s">
+        <v>14</v>
+      </c>
+      <c r="H77" t="s">
+        <v>346</v>
+      </c>
+      <c r="I77" t="s">
+        <v>160</v>
+      </c>
+      <c r="J77" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>246</v>
+      </c>
+      <c r="C78" t="s">
+        <v>347</v>
+      </c>
+      <c r="D78" t="s">
+        <v>348</v>
+      </c>
+      <c r="E78" t="s">
+        <v>349</v>
+      </c>
+      <c r="F78" t="s">
+        <v>13</v>
+      </c>
+      <c r="G78" t="s">
+        <v>14</v>
+      </c>
+      <c r="H78" t="s">
+        <v>350</v>
+      </c>
+      <c r="I78" t="s">
+        <v>160</v>
+      </c>
+      <c r="J78" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>246</v>
+      </c>
+      <c r="C79" t="s">
+        <v>351</v>
+      </c>
+      <c r="D79" t="s">
+        <v>352</v>
+      </c>
+      <c r="E79" t="s">
+        <v>353</v>
+      </c>
+      <c r="F79" t="s">
+        <v>13</v>
+      </c>
+      <c r="G79" t="s">
+        <v>14</v>
+      </c>
+      <c r="H79" t="s">
+        <v>354</v>
+      </c>
+      <c r="I79" t="s">
+        <v>160</v>
+      </c>
+      <c r="J79" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>246</v>
+      </c>
+      <c r="C80" t="s">
+        <v>355</v>
+      </c>
+      <c r="D80" t="s">
+        <v>356</v>
+      </c>
+      <c r="E80" t="s">
+        <v>357</v>
+      </c>
+      <c r="F80" t="s">
+        <v>13</v>
+      </c>
+      <c r="G80" t="s">
+        <v>14</v>
+      </c>
+      <c r="H80" t="s">
+        <v>358</v>
+      </c>
+      <c r="I80" t="s">
+        <v>160</v>
+      </c>
+      <c r="J80" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>246</v>
+      </c>
+      <c r="C81" t="s">
+        <v>359</v>
+      </c>
+      <c r="D81" t="s">
+        <v>360</v>
+      </c>
+      <c r="E81" t="s">
+        <v>361</v>
+      </c>
+      <c r="F81" t="s">
+        <v>13</v>
+      </c>
+      <c r="G81" t="s">
+        <v>14</v>
+      </c>
+      <c r="H81" t="s">
+        <v>362</v>
+      </c>
+      <c r="I81" t="s">
+        <v>160</v>
+      </c>
+      <c r="J81" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>82</v>
+      </c>
+      <c r="B82" t="s">
+        <v>253</v>
+      </c>
+      <c r="C82" t="s">
+        <v>254</v>
+      </c>
+      <c r="D82" t="s">
+        <v>255</v>
+      </c>
+      <c r="E82" t="s">
         <v>338</v>
       </c>
-      <c r="C77" t="s">
-        <v>339</v>
-      </c>
-      <c r="D77" t="s">
-        <v>340</v>
-      </c>
-      <c r="E77" t="s">
-        <v>341</v>
-      </c>
-      <c r="F77" t="s">
-        <v>36</v>
-      </c>
-      <c r="G77" t="s">
-        <v>175</v>
-      </c>
-      <c r="H77" t="s">
-        <v>342</v>
-      </c>
-      <c r="I77" t="s">
-        <v>175</v>
-      </c>
-      <c r="J77" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B79" t="s">
-        <v>343</v>
-      </c>
-      <c r="C79">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B80" t="s">
-        <v>344</v>
-      </c>
-      <c r="C80">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B81" t="s">
-        <v>345</v>
-      </c>
-      <c r="C81">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B82" t="s">
-        <v>346</v>
-      </c>
-      <c r="C82">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B83" t="s">
-        <v>347</v>
-      </c>
-      <c r="C83">
+      <c r="F82" t="s">
+        <v>31</v>
+      </c>
+      <c r="G82" t="s">
+        <v>132</v>
+      </c>
+      <c r="H82" t="s">
+        <v>256</v>
+      </c>
+      <c r="I82" t="s">
+        <v>132</v>
+      </c>
+      <c r="J82" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B84" t="s">
+        <v>257</v>
+      </c>
+      <c r="C84">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B85" t="s">
+        <v>258</v>
+      </c>
+      <c r="C85">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B86" t="s">
+        <v>259</v>
+      </c>
+      <c r="C86">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B87" t="s">
+        <v>260</v>
+      </c>
+      <c r="C87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B88" t="s">
+        <v>261</v>
+      </c>
+      <c r="C88">
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B84" t="s">
-        <v>348</v>
-      </c>
-      <c r="C84">
-        <v>8</v>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B89" t="s">
+        <v>262</v>
+      </c>
+      <c r="C89">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>